<commit_message>
Add Salesforce dependency caveat and conditional Opportunity #4
Salesforce represents 39.5% of vendor spend but we lack visibility into
whether this is over-provisioning or an operational necessity. Added:
- Caveat on Opportunity #1 flagging the information gap
- Conditional Opportunity #4: SaaS portfolio rationalization (~$60K-$100K)
  as fallback if Salesforce spend is operationally justified
- Savings range ($710K-$1.27M) shown across all artifacts
- Risk #5 in executive memo for Salesforce operational criticality
- Phase 0 (Salesforce dependency assessment) in implementation timeline

QA: 6/6 checks passed, spend reconciliation to $0.00 variance.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
+++ b/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -107,8 +107,32 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -216,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -319,29 +343,33 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21453,7 +21481,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="80" customWidth="1" style="33" min="1" max="1"/>
@@ -21538,109 +21566,170 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="42" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="42" t="inlineStr">
+        <is>
+          <t>IMPORTANT CAVEAT: We do not currently have sufficient information to determine why Salesforce spend represents 39.5% of total vendor costs. If this concentration exists because Salesforce is integral to revenue generation, core service delivery, or operational infrastructure (e.g., the company resells Salesforce solutions or uses it as a primary business platform), then aggressive cost reduction could directly harm the business. Stakeholder interviews with business unit leaders must be conducted before executing this opportunity. See Conditional Opportunity 4 below for an alternative savings path if Salesforce spend is operationally justified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="inlineStr">
         <is>
           <t>OPPORTUNITY 2: Office &amp; Facilities Consolidation</t>
         </is>
       </c>
-      <c r="B10" s="43" t="inlineStr">
+      <c r="B11" s="44" t="inlineStr">
         <is>
           <t>Est. Savings: $358,627/yr</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="44" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="45" t="inlineStr">
         <is>
           <t>Current Spend: $1,024,648 across 28 facility vendors</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>The organization uses multiple overlapping office and coworking providers across regions (TOG, WeWork, Innovent, GPT Space, Common Desk, Work Easy). This fragmentation prevents volume-based negotiation and creates administrative overhead managing 26 separate contracts.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="41" t="inlineStr">
         <is>
-          <t>Recommended Actions: (1) Map current headcount and space utilization per office location, (2) Consolidate to 2-3 preferred coworking/office providers with global coverage, (3) Negotiate master services agreements with volume discounts, (4) Implement space utilization monitoring to right-size footprint.</t>
+          <t>The organization uses multiple overlapping office and coworking providers across regions (TOG, WeWork, Innovent, GPT Space, Common Desk, Work Easy). This fragmentation prevents volume-based negotiation and creates administrative overhead managing 26 separate contracts.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="41" t="inlineStr">
         <is>
+          <t>Recommended Actions: (1) Map current headcount and space utilization per office location, (2) Consolidate to 2-3 preferred coworking/office providers with global coverage, (3) Negotiate master services agreements with volume discounts, (4) Implement space utilization monitoring to right-size footprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
           <t>Timeline: 2-3 months for analysis, 6-12 months for lease transitions as contracts expire.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="42" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="43" t="inlineStr">
         <is>
           <t>OPPORTUNITY 3: Elimination of Non-Essential Discretionary Spend</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
+      <c r="B17" s="44" t="inlineStr">
         <is>
           <t>Est. Savings: $131,461/yr</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="44" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="45" t="inlineStr">
         <is>
           <t>Current Spend: $154,660 across 77 vendors marked for termination</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="41" t="inlineStr">
-        <is>
-          <t>A significant portion of vendor spend is directed toward discretionary categories including corporate entertainment, restaurant venues, hotel bookings, catering, team building activities, and event services. While some of this spend supports culture, much can be reduced or eliminated.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="41" t="inlineStr">
         <is>
-          <t>Recommended Actions: (1) Implement a tiered approval process for discretionary spend, (2) Set quarterly budgets per department for entertainment and events, (3) Consolidate remaining event spend to 2-3 preferred vendors, (4) Eliminate one-off vendor relationships with no ongoing business need.</t>
+          <t>A significant portion of vendor spend is directed toward discretionary categories including corporate entertainment, restaurant venues, hotel bookings, catering, team building activities, and event services. While some of this spend supports culture, much can be reduced or eliminated.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>Timeline: Immediate for policy changes, 1-3 months for full implementation.</t>
+          <t>Recommended Actions: (1) Implement a tiered approval process for discretionary spend, (2) Set quarterly budgets per department for entertainment and events, (3) Consolidate remaining event spend to 2-3 preferred vendors, (4) Eliminate one-off vendor relationships with no ongoing business need.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="41" t="inlineStr">
         <is>
+          <t>Timeline: Immediate for policy changes, 1-3 months for full implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
           <t>Additional savings of $160,597 from consolidating professional services, insurance, and finance vendors through preferred supplier agreements and volume-based pricing.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="45" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="46" t="inlineStr">
+        <is>
+          <t>CONDITIONAL OPPORTUNITY 4: SaaS Portfolio Rationalization (Pending Salesforce Assessment)</t>
+        </is>
+      </c>
+      <c r="B24" s="47" t="inlineStr">
+        <is>
+          <t>Est. Savings: $59,566-$99,276/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>Current Spend: $397,105 across 47 non-Salesforce SaaS vendors</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>This opportunity is conditional: it applies if the Salesforce dependency assessment (see Opportunity 1 caveat) determines that Salesforce spend is operationally justified and cannot be materially reduced. We currently lack visibility into whether the 39.5% vendor spend concentration on Salesforce reflects over-provisioning or a legitimate operational dependency. This information must be gathered before committing to either Opportunity 1 or this alternative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>If Salesforce spend is confirmed as operationally critical, the savings focus shifts to rationalizing the remaining 47 non-Salesforce SaaS vendors ($397,105). This includes consolidating overlapping tools, eliminating underutilized licenses, and negotiating volume-based enterprise agreements across the broader SaaS portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>Required Actions Before Execution: (1) Conduct stakeholder interviews with business unit leaders to determine Salesforce's role in revenue generation and service delivery, (2) Map Salesforce product usage across departments, (3) Assess whether Salesforce spend is contractually locked or negotiable, (4) Based on findings, execute either Opportunity 1 (if optimizable) or this Opportunity 4 (if operationally critical).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>Timeline: 4-6 weeks for Salesforce dependency assessment, then 3-6 months for SaaS rationalization execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="48" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED ANNUAL SAVINGS</t>
         </is>
       </c>
-      <c r="B23" s="46" t="inlineStr">
+      <c r="B31" s="49" t="inlineStr">
         <is>
           <t>$1,274,130/yr</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="47" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
         <is>
           <t>This represents 16.2% of total vendor spend of $7,887,360</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="51" t="inlineStr">
+        <is>
+          <t>Conservative scenario (if Salesforce spend is operationally critical): $710,251/yr (9.0% of total spend) by replacing Opportunity 1 savings with Conditional Opportunity 4.</t>
         </is>
       </c>
     </row>
@@ -21685,7 +21774,7 @@
       <c r="B3" s="28" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="48" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>1. TOOLS USED</t>
         </is>
@@ -21693,7 +21782,7 @@
       <c r="B4" s="28" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>Primary Tool: Claude Code CLI (Anthropic) - AI-powered coding assistant for data analysis and automation</t>
         </is>
@@ -21717,7 +21806,7 @@
       <c r="B7" s="24" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="A9" s="43" t="inlineStr">
         <is>
           <t>2. CLASSIFICATION APPROACH</t>
         </is>
@@ -21752,7 +21841,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>3. DEPARTMENT TAXONOMY</t>
         </is>
@@ -21773,7 +21862,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>4. RECOMMENDATION FRAMEWORK</t>
         </is>
@@ -21801,7 +21890,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="A24" s="43" t="inlineStr">
         <is>
           <t>5. PROMPTS AND INSTRUCTIONS USED</t>
         </is>
@@ -21850,7 +21939,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="42" t="inlineStr">
+      <c r="A32" s="43" t="inlineStr">
         <is>
           <t>6. QUALITY CHECKS</t>
         </is>
@@ -21906,14 +21995,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="50" t="inlineStr">
+      <c r="A40" s="54" t="inlineStr">
         <is>
           <t>Result: 7/7 quality checks passed. Full report saved to quality-check/quality_check_report.txt</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="42" t="inlineStr">
+      <c r="A42" s="43" t="inlineStr">
         <is>
           <t>7. KEY FINDINGS SUMMARY</t>
         </is>
@@ -22035,14 +22124,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="110" customWidth="1" style="33" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>EXECUTIVE MEMO: Vendor Spend Optimization Recommendations</t>
         </is>
@@ -22050,7 +22139,7 @@
       <c r="B1" s="25" t="n"/>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="33">
-      <c r="A2" s="52" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>To: CEO / CFO  |  From: Marius de Villiers  |  Date: March 2026  |  Classification: Confidential</t>
         </is>
@@ -22062,7 +22151,7 @@
       <c r="B3" s="28" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="53" t="inlineStr">
+      <c r="A4" s="57" t="inlineStr">
         <is>
           <t>EXECUTIVE SUMMARY</t>
         </is>
@@ -22070,9 +22159,9 @@
       <c r="B4" s="28" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="inlineStr">
-        <is>
-          <t>Following a comprehensive analysis of 386 active vendor relationships totaling $7,887,360 in annual spend, I have identified three high-impact opportunities that could deliver estimated annual savings of $1,274,130. The analysis reveals significant vendor fragmentation, a critical single-vendor concentration risk, and substantial discretionary spend that can be rationalized. Beyond direct cost savings, this analysis establishes a vendor governance framework that can be scaled across the full enterprise to drive sustained procurement efficiency.</t>
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t>Following a comprehensive analysis of 386 active vendor relationships totaling $7,887,360 in annual spend, I have identified three high-impact opportunities plus one conditional opportunity that could deliver estimated annual savings of $710,251-$1,274,130 depending on the outcome of a Salesforce dependency assessment. The analysis reveals significant vendor fragmentation, a critical single-vendor concentration question, and substantial discretionary spend that can be rationalized. Beyond direct cost savings, this analysis establishes a vendor governance framework that can be scaled across the full enterprise to drive sustained procurement efficiency.</t>
         </is>
       </c>
       <c r="B5" s="28" t="n"/>
@@ -22082,7 +22171,7 @@
       <c r="B6" s="24" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="54" t="inlineStr">
+      <c r="A7" s="58" t="inlineStr">
         <is>
           <t>KEY FINDINGS</t>
         </is>
@@ -22092,7 +22181,7 @@
     <row r="8">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>1. CONCENTRATION RISK: Salesforce represents $3,117,226 (39.5% of total spend). This single-vendor dependency creates pricing leverage imbalance and operational risk.</t>
+          <t>1. CONCENTRATION QUESTION: Salesforce represents $3,117,226 (39.5% of total spend). We do not currently have visibility into whether this concentration reflects over-provisioning or an operationally justified dependency (e.g., revenue-generating platform, core service delivery tool). A stakeholder assessment is required before determining if this represents a cost-reduction opportunity or a strategic investment that should be protected.</t>
         </is>
       </c>
     </row>
@@ -22118,14 +22207,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="45" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>RECOMMENDED ACTIONS AND TIMELINE</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="54" t="inlineStr">
         <is>
           <t>Phase 1 - Quick Wins (0-3 months):</t>
         </is>
@@ -22153,7 +22242,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="50" t="inlineStr">
+      <c r="A19" s="54" t="inlineStr">
         <is>
           <t>Phase 2 - Strategic Consolidation (3-6 months):</t>
         </is>
@@ -22181,7 +22270,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="50" t="inlineStr">
+      <c r="A24" s="54" t="inlineStr">
         <is>
           <t>Phase 3 - Enterprise Renegotiation (6-12 months):</t>
         </is>
@@ -22209,7 +22298,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="45" t="inlineStr">
+      <c r="A29" s="48" t="inlineStr">
         <is>
           <t>IMPLEMENTATION RISKS AND MITIGATION</t>
         </is>
@@ -22243,50 +22332,57 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="45" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>Risk 5: Salesforce spend may be operationally critical. If Salesforce is integral to revenue generation or core service delivery, reducing spend could directly harm the business. Mitigation: Conduct stakeholder interviews before executing Opportunity 1; if spend is justified, pivot to Conditional Opportunity 4 (SaaS portfolio rationalization) for alternative savings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="48" t="inlineStr">
         <is>
           <t>EXPECTED OUTCOMES</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="41" t="inlineStr">
-        <is>
-          <t>- Total estimated annual savings: $1,274,130 (16.2% of total spend)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
         <is>
-          <t>- Vendor count reduction: From 386 to approximately 273 active vendors</t>
+          <t>- Total estimated annual savings: $710,251-$1,274,130 (9.0%-16.2% of total spend), depending on outcome of Salesforce dependency assessment</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
         <is>
-          <t>- Improved procurement governance and spend visibility across all departments</t>
+          <t>- Vendor count reduction: From 386 to approximately 273 active vendors</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
         <is>
-          <t>- Reduced single-vendor concentration risk through strategic diversification</t>
+          <t>- Improved procurement governance and spend visibility across all departments</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="41" t="inlineStr">
         <is>
-          <t>- Scalable vendor governance methodology applicable across all business units and spend categories</t>
+          <t>- Reduced single-vendor concentration risk through strategic diversification</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>- Scalable vendor governance methodology applicable across all business units and spend categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="41" t="inlineStr">
         <is>
           <t>Note: This analysis covers $7.9M in identified vendor spend. Applying the same methodology across all procurement categories of a $1B enterprise could yield 10-15x these savings.</t>
         </is>

</xml_diff>

<commit_message>
Soften Salesforce caveat language to avoid asserting operational criticality
Changed all Salesforce dependency language from assertions ("is integral",
"is operationally critical", "the company resells") to possibilities
("may reflect", "it is possible that", "could indicate"). The caveat
now frames the information gap as something to investigate rather than
claiming to know why the concentration exists.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
+++ b/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
@@ -21569,7 +21569,7 @@
     <row r="9">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>IMPORTANT CAVEAT: We do not currently have sufficient information to determine why Salesforce spend represents 39.5% of total vendor costs. If this concentration exists because Salesforce is integral to revenue generation, core service delivery, or operational infrastructure (e.g., the company resells Salesforce solutions or uses it as a primary business platform), then aggressive cost reduction could directly harm the business. Stakeholder interviews with business unit leaders must be conducted before executing this opportunity. See Conditional Opportunity 4 below for an alternative savings path if Salesforce spend is operationally justified.</t>
+          <t>IMPORTANT CAVEAT: We do not currently have sufficient information to determine why Salesforce spend represents 39.5% of total vendor costs. It is possible that this concentration reflects a deeper operational dependency — for example, Salesforce may play a role in revenue generation, service delivery, or core business operations. If that were the case, aggressive cost reduction could risk harming the business. We recommend stakeholder interviews with business unit leaders to understand the nature of this spend before executing this opportunity. See Conditional Opportunity 4 below for an alternative savings path should the assessment reveal that Salesforce spend cannot be materially reduced.</t>
         </is>
       </c>
     </row>
@@ -21682,21 +21682,21 @@
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>This opportunity is conditional: it applies if the Salesforce dependency assessment (see Opportunity 1 caveat) determines that Salesforce spend is operationally justified and cannot be materially reduced. We currently lack visibility into whether the 39.5% vendor spend concentration on Salesforce reflects over-provisioning or a legitimate operational dependency. This information must be gathered before committing to either Opportunity 1 or this alternative.</t>
+          <t>This opportunity is conditional: it applies if the Salesforce dependency assessment (see Opportunity 1 caveat) reveals that Salesforce spend cannot be materially reduced. We currently lack visibility into whether the 39.5% vendor spend concentration on Salesforce reflects over-provisioning or a deeper operational need. This information must be gathered before committing to either Opportunity 1 or this alternative.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>If Salesforce spend is confirmed as operationally critical, the savings focus shifts to rationalizing the remaining 47 non-Salesforce SaaS vendors ($397,105). This includes consolidating overlapping tools, eliminating underutilized licenses, and negotiating volume-based enterprise agreements across the broader SaaS portfolio.</t>
+          <t>If the assessment indicates that Salesforce spend cannot be materially reduced, the savings focus shifts to rationalizing the remaining 47 non-Salesforce SaaS vendors ($397,105). This includes consolidating overlapping tools, eliminating underutilized licenses, and negotiating volume-based enterprise agreements across the broader SaaS portfolio.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="41" t="inlineStr">
         <is>
-          <t>Required Actions Before Execution: (1) Conduct stakeholder interviews with business unit leaders to determine Salesforce's role in revenue generation and service delivery, (2) Map Salesforce product usage across departments, (3) Assess whether Salesforce spend is contractually locked or negotiable, (4) Based on findings, execute either Opportunity 1 (if optimizable) or this Opportunity 4 (if operationally critical).</t>
+          <t>Required Actions Before Execution: (1) Conduct stakeholder interviews with business unit leaders to determine the business rationale behind the Salesforce spend concentration, (2) Map Salesforce product usage across departments, (3) Assess whether Salesforce spend is contractually locked or negotiable, (4) Based on findings, execute either Opportunity 1 (if spend is optimizable) or this Opportunity 4 (if spend cannot be reduced).</t>
         </is>
       </c>
     </row>
@@ -21729,7 +21729,7 @@
     <row r="33">
       <c r="A33" s="51" t="inlineStr">
         <is>
-          <t>Conservative scenario (if Salesforce spend is operationally critical): $710,251/yr (9.0% of total spend) by replacing Opportunity 1 savings with Conditional Opportunity 4.</t>
+          <t>Conservative scenario (if Salesforce spend cannot be materially reduced): $710,251/yr (9.0% of total spend) by replacing Opportunity 1 savings with Conditional Opportunity 4.</t>
         </is>
       </c>
     </row>
@@ -22181,7 +22181,7 @@
     <row r="8">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>1. CONCENTRATION QUESTION: Salesforce represents $3,117,226 (39.5% of total spend). We do not currently have visibility into whether this concentration reflects over-provisioning or an operationally justified dependency (e.g., revenue-generating platform, core service delivery tool). A stakeholder assessment is required before determining if this represents a cost-reduction opportunity or a strategic investment that should be protected.</t>
+          <t>1. CONCENTRATION QUESTION: Salesforce represents $3,117,226 (39.5% of total spend). We do not currently have visibility into why this concentration is so high. It may reflect over-provisioning, or it could indicate a deeper operational dependency. A stakeholder assessment is required before determining whether this represents a cost-reduction opportunity or spend that should be protected.</t>
         </is>
       </c>
     </row>
@@ -22335,7 +22335,7 @@
     <row r="34">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t>Risk 5: Salesforce spend may be operationally critical. If Salesforce is integral to revenue generation or core service delivery, reducing spend could directly harm the business. Mitigation: Conduct stakeholder interviews before executing Opportunity 1; if spend is justified, pivot to Conditional Opportunity 4 (SaaS portfolio rationalization) for alternative savings.</t>
+          <t>Risk 5: Salesforce spend concentration is not yet understood. It is possible that the 39.5% concentration reflects a deeper operational need, in which case reducing spend could have unintended consequences. Mitigation: Conduct stakeholder interviews to understand the business rationale before executing Opportunity 1; if spend cannot be reduced, pivot to Conditional Opportunity 4 (SaaS portfolio rationalization).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final audit fixes: numbering consistency, Phase 0 in Excel, methodology updates
- Fix executive_memo.md: "Conditional Opportunity 5" → "4" (2 places)
- Fix methodology.md: add Salesforce caveat, savings range, conditional opp, fix duplicate numbering
- Fix process_all.py: add Phase 0 (Salesforce Assessment) to Excel exec memo tab
- Fix process_all.py: remove "concentration risk" from expected outcomes
- Fix change_log.md: corrupted \B → $1B, add Salesforce caveat change entries
- Fix data_dictionary.md: mention conditional opportunity in Top 3 tab description
- Regenerated Excel and QA report (6/6 PASS)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
+++ b/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
@@ -22124,7 +22124,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="110" customWidth="1" style="33" min="1" max="1"/>
@@ -22216,173 +22216,201 @@
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>Phase 1 - Quick Wins (0-3 months):</t>
+          <t>Phase 0 - Salesforce Dependency Assessment (0-6 weeks):</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>- Implement discretionary spend approval process and per-department budgets for events/entertainment</t>
+          <t>- Conduct stakeholder interviews with business unit leaders to understand why Salesforce represents 39.5% of vendor spend</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>- Begin termination of one-off vendor relationships with no ongoing business justification</t>
+          <t>- Map Salesforce product usage across all departments to determine if it is a cost center (optimizable) or operational necessity</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="41" t="inlineStr">
         <is>
-          <t>- Initiate Salesforce license utilization audit to identify dormant or underused licenses</t>
+          <t>- Based on findings, execute either Opportunity 1 (Salesforce optimization) or Conditional Opportunity 4 (SaaS rationalization)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>Phase 2 - Strategic Consolidation (3-6 months):</t>
+          <t>Phase 1 - Quick Wins (0-3 months):</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>- Consolidate office/coworking vendors to 2-3 preferred providers with master agreements</t>
+          <t>- Implement discretionary spend approval process and per-department budgets for events/entertainment</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="41" t="inlineStr">
         <is>
-          <t>- Rationalize insurance providers and consolidate to regional preferred brokers</t>
+          <t>- Begin termination of one-off vendor relationships with no ongoing business justification</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="41" t="inlineStr">
         <is>
-          <t>- Consolidate recruitment agencies to 3-4 strategic partners with preferred pricing</t>
+          <t>- Initiate Salesforce license utilization audit to identify dormant or underused licenses</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>Phase 3 - Enterprise Renegotiation (6-12 months):</t>
+          <t>Phase 2 - Strategic Consolidation (3-6 months):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>- Renegotiate Salesforce enterprise agreement leveraging license audit findings and competitive alternatives</t>
+          <t>- Consolidate office/coworking vendors to 2-3 preferred providers with master agreements</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>- Implement vendor management platform for ongoing spend visibility and contract lifecycle management</t>
+          <t>- Rationalize insurance providers and consolidate to regional preferred brokers</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>- Establish quarterly vendor performance reviews for top 20 vendors by spend</t>
+          <t>- Consolidate recruitment agencies to 3-4 strategic partners with preferred pricing</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="48" t="inlineStr">
-        <is>
-          <t>IMPLEMENTATION RISKS AND MITIGATION</t>
+      <c r="A29" s="54" t="inlineStr">
+        <is>
+          <t>Phase 3 - Enterprise Renegotiation (6-12 months):</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
-          <t>Risk 1: Salesforce renegotiation timeline. Mitigation: Begin audit immediately; secure competitive quotes from Microsoft Dynamics and HubSpot as leverage.</t>
+          <t>- Renegotiate Salesforce enterprise agreement leveraging license audit findings and competitive alternatives</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t>Risk 2: Office lease lock-in periods. Mitigation: Map all lease expiry dates; target consolidation as each lease comes up for renewal.</t>
+          <t>- Implement vendor management platform for ongoing spend visibility and contract lifecycle management</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="41" t="inlineStr">
         <is>
-          <t>Risk 3: Employee morale impact from reducing perks/events. Mitigation: Maintain core team-building budget; optimize rather than eliminate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="41" t="inlineStr">
-        <is>
-          <t>Risk 4: Operational disruption during vendor transitions. Mitigation: Phase transitions with overlap periods; assign a dedicated project manager.</t>
+          <t>- Establish quarterly vendor performance reviews for top 20 vendors by spend</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="41" t="inlineStr">
-        <is>
-          <t>Risk 5: Salesforce spend concentration is not yet understood. It is possible that the 39.5% concentration reflects a deeper operational need, in which case reducing spend could have unintended consequences. Mitigation: Conduct stakeholder interviews to understand the business rationale before executing Opportunity 1; if spend cannot be reduced, pivot to Conditional Opportunity 4 (SaaS portfolio rationalization).</t>
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <t>IMPLEMENTATION RISKS AND MITIGATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>Risk 1: Salesforce renegotiation timeline. Mitigation: Begin audit immediately; secure competitive quotes from Microsoft Dynamics and HubSpot as leverage.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="48" t="inlineStr">
-        <is>
-          <t>EXPECTED OUTCOMES</t>
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>Risk 2: Office lease lock-in periods. Mitigation: Map all lease expiry dates; target consolidation as each lease comes up for renewal.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
         <is>
-          <t>- Total estimated annual savings: $710,251-$1,274,130 (9.0%-16.2% of total spend), depending on outcome of Salesforce dependency assessment</t>
+          <t>Risk 3: Employee morale impact from reducing perks/events. Mitigation: Maintain core team-building budget; optimize rather than eliminate.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
         <is>
-          <t>- Vendor count reduction: From 386 to approximately 273 active vendors</t>
+          <t>Risk 4: Operational disruption during vendor transitions. Mitigation: Phase transitions with overlap periods; assign a dedicated project manager.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
         <is>
-          <t>- Improved procurement governance and spend visibility across all departments</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="41" t="inlineStr">
-        <is>
-          <t>- Reduced single-vendor concentration risk through strategic diversification</t>
+          <t>Risk 5: Salesforce spend concentration is not yet understood. It is possible that the 39.5% concentration reflects a deeper operational need, in which case reducing spend could have unintended consequences. Mitigation: Conduct stakeholder interviews to understand the business rationale before executing Opportunity 1; if spend cannot be reduced, pivot to Conditional Opportunity 4 (SaaS portfolio rationalization).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="41" t="inlineStr">
-        <is>
-          <t>- Scalable vendor governance methodology applicable across all business units and spend categories</t>
+      <c r="A41" s="48" t="inlineStr">
+        <is>
+          <t>EXPECTED OUTCOMES</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>- Total estimated annual savings: $710,251-$1,274,130 (9.0%-16.2% of total spend), depending on outcome of Salesforce dependency assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>- Vendor count reduction: From 386 to approximately 273 active vendors</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="41" t="inlineStr">
+        <is>
+          <t>- Improved procurement governance and spend visibility across all departments</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>- Reduced single-vendor concentration through strategic diversification</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>- Scalable vendor governance methodology applicable across all business units and spend categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="41" t="inlineStr">
         <is>
           <t>Note: This analysis covers $7.9M in identified vendor spend. Applying the same methodology across all procurement categories of a $1B enterprise could yield 10-15x these savings.</t>
         </is>

</xml_diff>

<commit_message>
Fix remaining assertive Salesforce language and format consistency
- "extreme concentration creates" → "concentration may represent"
- "critical single-vendor concentration" → "requiring assessment"
- Convert .format() to f-string for consistency

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
+++ b/03_outputs/Vendor Analysis Assessment - Marius de Villiers.xlsx
@@ -21542,7 +21542,7 @@
     <row r="6">
       <c r="A6" s="40" t="inlineStr">
         <is>
-          <t>Salesforce represents the single largest vendor relationship at nearly 40% of total spend. This extreme concentration creates both significant risk and optimization opportunity. A structured license audit typically reveals 15-25% of licenses are underutilized or dormant. Given the scale of this relationship, even modest optimization yields substantial absolute savings.</t>
+          <t>Salesforce represents the single largest vendor relationship at nearly 40% of total spend. This concentration may represent both significant risk and optimization opportunity. A structured license audit typically reveals 15-25% of licenses are underutilized or dormant. Given the scale of this relationship, even modest optimization yields substantial absolute savings.</t>
         </is>
       </c>
       <c r="B6" s="24" t="n"/>
@@ -22161,7 +22161,7 @@
     <row r="5">
       <c r="A5" s="53" t="inlineStr">
         <is>
-          <t>Following a comprehensive analysis of 386 active vendor relationships totaling $7,887,360 in annual spend, I have identified three high-impact opportunities plus one conditional opportunity that could deliver estimated annual savings of $710,251-$1,274,130 depending on the outcome of a Salesforce dependency assessment. The analysis reveals significant vendor fragmentation, a critical single-vendor concentration question, and substantial discretionary spend that can be rationalized. Beyond direct cost savings, this analysis establishes a vendor governance framework that can be scaled across the full enterprise to drive sustained procurement efficiency.</t>
+          <t>Following a comprehensive analysis of 386 active vendor relationships totaling $7,887,360 in annual spend, I have identified three high-impact opportunities plus one conditional opportunity that could deliver estimated annual savings of $710,251-$1,274,130 depending on the outcome of a Salesforce dependency assessment. The analysis reveals significant vendor fragmentation, a single-vendor concentration question requiring assessment, and substantial discretionary spend that can be rationalized. Beyond direct cost savings, this analysis establishes a vendor governance framework that can be scaled across the full enterprise to drive sustained procurement efficiency.</t>
         </is>
       </c>
       <c r="B5" s="28" t="n"/>

</xml_diff>